<commit_message>
chore(data): update prepod_user_list.xlsx [2026-08-25T01:56:53.163Z]
</commit_message>
<xml_diff>
--- a/prepod_user_list.xlsx
+++ b/prepod_user_list.xlsx
@@ -502,7 +502,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -812,9 +812,32 @@
         <v>{"walletAddress":"mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9"}</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-08-25T01:56:52.144Z</v>
+      </c>
+      <c r="B14" t="str">
+        <v>user.login</v>
+      </c>
+      <c r="C14" t="str">
+        <v>7ca8a6ec-25cc-4dcd-92f6-39ef7c83b22a</v>
+      </c>
+      <c r="D14" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Sujeet Kulkarni</v>
+      </c>
+      <c r="F14" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+      <c r="G14" t="str">
+        <v>{}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(data): update prepod_user_list.xlsx [2026-08-25T01:59:02.183Z]
</commit_message>
<xml_diff>
--- a/prepod_user_list.xlsx
+++ b/prepod_user_list.xlsx
@@ -502,7 +502,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -835,16 +835,62 @@
         <v>{}</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-08-25T01:57:19.644Z</v>
+      </c>
+      <c r="B15" t="str">
+        <v>user.wallet_linked</v>
+      </c>
+      <c r="C15" t="str">
+        <v>7ca8a6ec-25cc-4dcd-92f6-39ef7c83b22a</v>
+      </c>
+      <c r="D15" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Sujeet Kulkarni</v>
+      </c>
+      <c r="F15" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+      <c r="G15" t="str">
+        <v>{"walletAddress":"mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9"}</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-08-25T01:59:01.283Z</v>
+      </c>
+      <c r="B16" t="str">
+        <v>user.login</v>
+      </c>
+      <c r="C16" t="str">
+        <v>7ca8a6ec-25cc-4dcd-92f6-39ef7c83b22a</v>
+      </c>
+      <c r="D16" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Sujeet Kulkarni</v>
+      </c>
+      <c r="F16" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+      <c r="G16" t="str">
+        <v>{}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J15"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1210,9 +1256,137 @@
         <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>0fcd26c3-0c2b-4184-8bf5-3d684bb1254e</v>
+      </c>
+      <c r="B12" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PAN</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E12" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F12" t="str">
+        <v>e3ce454539d781cc03dfb4b4bf82fa5ce0100ef95d7d771a871c61070a67d6c2</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-08-25T01:57:26.918Z</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2027-08-25T01:57:26.917Z</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>47329955-b236-4fb4-a636-2273f7b5191b</v>
+      </c>
+      <c r="B13" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C13" t="str">
+        <v>AADHAAR</v>
+      </c>
+      <c r="D13" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E13" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F13" t="str">
+        <v>fcb53e3dffa4715f9af921314d9756132adc256c3185a8e8cd4f882c08dcd7b6</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-08-25T01:57:27.719Z</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2027-08-25T01:57:27.718Z</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>9faecfb8-bc38-4dca-9bf3-8a2b7f5103ec</v>
+      </c>
+      <c r="B14" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C14" t="str">
+        <v>AGE</v>
+      </c>
+      <c r="D14" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E14" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F14" t="str">
+        <v>c4896bbc1fe53295a179344e3040ef1835dd5e69c644f138827a3df4febff0bf</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-08-25T01:57:28.315Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2027-08-25T01:57:28.313Z</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>fd5a55e0-288f-4ddb-96c8-a26f74e982fb</v>
+      </c>
+      <c r="B15" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C15" t="str">
+        <v>RESIDENCY</v>
+      </c>
+      <c r="D15" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E15" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F15" t="str">
+        <v>869ca46d6d4ad38265709c0edcccff1e489f9a86c6a87343a460f1243b0126b1</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-08-25T01:57:28.932Z</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2027-08-25T01:57:28.931Z</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): update prepod_user_list.xlsx [2026-08-25T14:18:01.068Z]
</commit_message>
<xml_diff>
--- a/prepod_user_list.xlsx
+++ b/prepod_user_list.xlsx
@@ -502,7 +502,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -881,16 +881,39 @@
         <v>{}</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-08-25T14:17:56.552Z</v>
+      </c>
+      <c r="B17" t="str">
+        <v>user.login</v>
+      </c>
+      <c r="C17" t="str">
+        <v>7ca8a6ec-25cc-4dcd-92f6-39ef7c83b22a</v>
+      </c>
+      <c r="D17" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Sujeet Kulkarni</v>
+      </c>
+      <c r="F17" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+      <c r="G17" t="str">
+        <v>{}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J19"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1267,7 +1290,7 @@
         <v>PAN</v>
       </c>
       <c r="D12" t="str">
-        <v>ACTIVE</v>
+        <v>REVOKED</v>
       </c>
       <c r="E12" t="str">
         <v>SyntheticIdentityProvider</v>
@@ -1282,7 +1305,7 @@
         <v>2027-08-25T01:57:26.917Z</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>2026-08-25T01:59:29.680Z</v>
       </c>
       <c r="J12" t="str">
         <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
@@ -1299,7 +1322,7 @@
         <v>AADHAAR</v>
       </c>
       <c r="D13" t="str">
-        <v>ACTIVE</v>
+        <v>REVOKED</v>
       </c>
       <c r="E13" t="str">
         <v>SyntheticIdentityProvider</v>
@@ -1314,7 +1337,7 @@
         <v>2027-08-25T01:57:27.718Z</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>2026-08-25T01:59:28.680Z</v>
       </c>
       <c r="J13" t="str">
         <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
@@ -1331,7 +1354,7 @@
         <v>AGE</v>
       </c>
       <c r="D14" t="str">
-        <v>ACTIVE</v>
+        <v>REVOKED</v>
       </c>
       <c r="E14" t="str">
         <v>SyntheticIdentityProvider</v>
@@ -1346,7 +1369,7 @@
         <v>2027-08-25T01:57:28.313Z</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>2026-08-25T01:59:30.748Z</v>
       </c>
       <c r="J14" t="str">
         <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
@@ -1363,7 +1386,7 @@
         <v>RESIDENCY</v>
       </c>
       <c r="D15" t="str">
-        <v>ACTIVE</v>
+        <v>REVOKED</v>
       </c>
       <c r="E15" t="str">
         <v>SyntheticIdentityProvider</v>
@@ -1378,15 +1401,143 @@
         <v>2027-08-25T01:57:28.931Z</v>
       </c>
       <c r="I15" t="str">
+        <v>2026-08-25T01:59:28.127Z</v>
+      </c>
+      <c r="J15" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>34dec55f-77a1-44f3-b19c-cceae4bcb5fc</v>
+      </c>
+      <c r="B16" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PAN</v>
+      </c>
+      <c r="D16" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E16" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F16" t="str">
+        <v>29d9e130511997b08981c88dd25538862bb148310517a82c19e057fd0a524861</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-08-25T01:59:31.686Z</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2027-08-25T01:59:31.685Z</v>
+      </c>
+      <c r="I16" t="str">
         <v/>
       </c>
-      <c r="J15" t="str">
+      <c r="J16" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>a25fa3ba-313e-4868-a453-87597caa334c</v>
+      </c>
+      <c r="B17" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C17" t="str">
+        <v>AADHAAR</v>
+      </c>
+      <c r="D17" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E17" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F17" t="str">
+        <v>5d1e79bd3bf0d5903d89afd7d67aae0e5d3d1561e9cb4cb31704ea31c1a3e6f5</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-08-25T01:59:32.344Z</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2027-08-25T01:59:32.343Z</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>7115421c-e4c0-4201-962a-811695e1fa1d</v>
+      </c>
+      <c r="B18" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C18" t="str">
+        <v>AGE</v>
+      </c>
+      <c r="D18" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E18" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F18" t="str">
+        <v>f5718485ea8de9008a3a8536caad03e4faaa086fa30850ba8c71ad3f480702bf</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-08-25T01:59:32.840Z</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2027-08-25T01:59:32.839Z</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>68e380ce-792a-46d3-9d62-399152a6e5f8</v>
+      </c>
+      <c r="B19" t="str">
+        <v>sujxxtxz._</v>
+      </c>
+      <c r="C19" t="str">
+        <v>RESIDENCY</v>
+      </c>
+      <c r="D19" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="E19" t="str">
+        <v>SyntheticIdentityProvider</v>
+      </c>
+      <c r="F19" t="str">
+        <v>a2bd6acc994145e8d5f4f6101147f1b7c3856ca9f46f021a8b1fe9a0a485cb07</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-08-25T01:59:33.277Z</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2027-08-25T01:59:33.276Z</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
         <v>mn_shield-addr_preprod1ftegpp6f68ttuc95y3mlx4zk7zr370kjl3denkd2nf8sfkh7n4nl5r2vkju8gd3tgjqw0v2wxmc2r77j83cpwfs36pckq8l9drn5h0cpm9gw9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>